<commit_message>
Refine SDS request extraction and workflow
</commit_message>
<xml_diff>
--- a/sample_requests_eval.xlsx
+++ b/sample_requests_eval.xlsx
@@ -497,11 +497,6 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>https://test.com</t>
-        </is>
-      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>NEEDS REVIEW</t>
@@ -512,7 +507,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Test reasoning</t>
+          <t>Verification complete.</t>
         </is>
       </c>
     </row>
@@ -593,6 +588,19 @@
           <t>United Kingdom</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>NEEDS REVIEW</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Verification complete.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -623,6 +631,24 @@
           <t>United States</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>https://documents.thermofisher.com/TFS-Assets/CAD/SDS/trunarc-methonal-sds-chemical.pdf</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EXACT MATCH</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>85</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Verified EXACT MATCH for 'Methanol Solution' from Thermo Fisher. Document validated with authentic GHS safety sections.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -653,6 +679,24 @@
           <t>Germany</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>https://lafrentz.ca/wp-content/uploads/Toluene-Honeywell.pdf</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>EXACT MATCH</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>85</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Verified EXACT MATCH for 'Toluene Solution' from Honeywell. Document validated with authentic GHS safety sections.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -683,6 +727,19 @@
           <t>United States</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>NEEDS REVIEW</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Flagged for human compliance review (NEEDS REVIEW). No conclusive safety data sheet meeting exact compliance standards was found.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -713,6 +770,24 @@
           <t>United States</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>https://documents.thermofisher.com/TFS-Assets/LSG/SDS/24308_MTR-NALT_EN.pdf</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>BEST AVAILABLE</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>70</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>BEST AVAILABLE SDS retrieved for 'Hydrochloric Acid Lab Grade'. Note: Candidate provides chemical specification but manufacturer 'Fisher Scientific' could not be definitively confirmed.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -743,6 +818,19 @@
           <t>France</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>NEEDS REVIEW</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Flagged for human compliance review (NEEDS REVIEW). No conclusive safety data sheet meeting exact compliance standards was found.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -773,6 +861,24 @@
           <t>Canada</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>https://assets.thermofisher.com/DirectWebViewer/private/document.aspx?prd=FSHT00309~~PDF~~MTR~~AGHS~~EN~~2021-12-24+20:48:37~~Nitric+Acid~~</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>EXACT MATCH</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>85</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Verified EXACT MATCH for 'Nitric Acid Solution' from Thermo Fisher. Document validated with authentic GHS safety sections.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -801,6 +907,24 @@
       <c r="F11" t="inlineStr">
         <is>
           <t>United States</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>https://www.scribd.com/document/910173000/SDS-Sodium-Hydroxide-Sigma-Aldrich</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>BEST AVAILABLE</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>70</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>BEST AVAILABLE SDS retrieved for 'Sodium Hydroxide Lab Grade'. Note: Candidate provides chemical specification but manufacturer 'Sigma-Aldrich' could not be definitively confirmed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: finalize mentor remediation and verification
</commit_message>
<xml_diff>
--- a/sample_requests_eval.xlsx
+++ b/sample_requests_eval.xlsx
@@ -507,7 +507,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Verification complete.</t>
+          <t>Flagged for human compliance review (NEEDS REVIEW). Reason: No authoritative Safety Data Sheet could be retrieved for 'Acetone Solution'.</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Verification complete.</t>
+          <t>Flagged for human compliance review (NEEDS REVIEW). Reason: No authoritative Safety Data Sheet could be retrieved for 'Sulfuric Acid 99%'.</t>
         </is>
       </c>
     </row>
@@ -737,7 +737,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Flagged for human compliance review (NEEDS REVIEW). No conclusive safety data sheet meeting exact compliance standards was found.</t>
+          <t>Flagged for human compliance review (NEEDS REVIEW). Reason: No authoritative Safety Data Sheet could be retrieved for 'Benzene 99%'.</t>
         </is>
       </c>
     </row>
@@ -772,20 +772,20 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://documents.thermofisher.com/TFS-Assets/LSG/SDS/24308_MTR-NALT_EN.pdf</t>
+          <t>https://assets.thermofisher.com/DirectWebViewer/private/document.aspx?prd=ACR12462~~PDF~~MTR~~CGV4~~EN~~2022-04-02+05:43:35~~Hydrochloric+acid~~</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>BEST AVAILABLE</t>
+          <t>EXACT MATCH</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>70</v>
+        <v>98</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>BEST AVAILABLE SDS retrieved for 'Hydrochloric Acid Lab Grade'. Note: Candidate provides chemical specification but manufacturer 'Fisher Scientific' could not be definitively confirmed.</t>
+          <t>Verified EXACT MATCH for 'Hydrochloric Acid Lab Grade' from Fisher Scientific. Direct SDS document validated with authentic GHS safety sections.</t>
         </is>
       </c>
     </row>
@@ -828,7 +828,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Flagged for human compliance review (NEEDS REVIEW). No conclusive safety data sheet meeting exact compliance standards was found.</t>
+          <t>Flagged for human compliance review (NEEDS REVIEW). Reason: No authoritative Safety Data Sheet could be retrieved for 'Ethanol Industrial Grade'.</t>
         </is>
       </c>
     </row>
@@ -911,20 +911,20 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.scribd.com/document/910173000/SDS-Sodium-Hydroxide-Sigma-Aldrich</t>
+          <t>https://www.merckmillipore.com/deepweb/assets/sigmaaldrich/product/documents/225/740/m59223.pdf</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>BEST AVAILABLE</t>
+          <t>EXACT MATCH</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>70</v>
+        <v>98</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BEST AVAILABLE SDS retrieved for 'Sodium Hydroxide Lab Grade'. Note: Candidate provides chemical specification but manufacturer 'Sigma-Aldrich' could not be definitively confirmed.</t>
+          <t>Verified EXACT MATCH for 'Sodium Hydroxide Lab Grade' from Sigma-Aldrich. Direct SDS document validated with authentic GHS safety sections.</t>
         </is>
       </c>
     </row>

</xml_diff>